<commit_message>
Separate 2024 sales and return adjustment imports; document lookup fix
</commit_message>
<xml_diff>
--- a/outputs/btl-bhh-20261026/LIEN_KET_BTL_BHH_2024.xlsx
+++ b/outputs/btl-bhh-20261026/LIEN_KET_BTL_BHH_2024.xlsx
@@ -2,10 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi tiet BTL-BHH" sheetId="1" r:id="R4e0e066759f243c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phieu BTL" sheetId="2" r:id="Rec254daae08d43f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thong tin" sheetId="3" r:id="R4afe1d6776354124"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chua co BHH" sheetId="4" r:id="Rb9c1674da35d4522"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi tiet BTL-BHH" sheetId="1" r:id="R973c4af51ca04267"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phieu BTL" sheetId="2" r:id="Rf74ecdd4e1614b26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thong tin" sheetId="3" r:id="Rcdffad4afbf34c8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,13 +15,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
     <x:numFmt numFmtId="201" formatCode="@"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.00########"/>
     <x:numFmt numFmtId="203" formatCode="#,##0;[Red](#,##0);0"/>
     <x:numFmt numFmtId="204" formatCode="#,##0.00"/>
-    <x:numFmt numFmtId="205" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="3">
     <x:font>
@@ -40,7 +38,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -50,11 +48,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF24435C"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -70,7 +63,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -105,12 +98,6 @@
     </x:xf>
     <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -172,7 +159,7 @@
     <x:tableColumn id="2" name="Ngày hạch toán"/>
     <x:tableColumn id="3" name="Khách hàng"/>
     <x:tableColumn id="4" name="Số dòng hàng"/>
-    <x:tableColumn id="5" name="BHH gốc trên AMIS"/>
+    <x:tableColumn id="5" name="BHH gốc đã xác định"/>
     <x:tableColumn id="6" name="Số lượng trả"/>
     <x:tableColumn id="7" name="Tiền hàng trả (VND)"/>
     <x:tableColumn id="8" name="VAT trả (VND)"/>
@@ -191,32 +178,6 @@
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Nội dung"/>
     <x:tableColumn id="2" name="Giá trị"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="UVG_4_BTL" displayName="UVG_4_BTL" ref="A1:Q2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:Q2"/>
-  <x:tableColumns count="17">
-    <x:tableColumn id="1" name="Số phiếu BTL"/>
-    <x:tableColumn id="2" name="Ngày hạch toán"/>
-    <x:tableColumn id="3" name="BHH gốc đang trống"/>
-    <x:tableColumn id="4" name="Dòng BTL"/>
-    <x:tableColumn id="5" name="Mã hàng"/>
-    <x:tableColumn id="6" name="Tên hàng"/>
-    <x:tableColumn id="7" name="ĐVT"/>
-    <x:tableColumn id="8" name="Số lượng trả"/>
-    <x:tableColumn id="9" name="Đơn giá (VND)"/>
-    <x:tableColumn id="10" name="Tiền hàng trả (VND)"/>
-    <x:tableColumn id="11" name="Thuế suất GTGT (%)"/>
-    <x:tableColumn id="12" name="Tiền thuế GTGT (VND)"/>
-    <x:tableColumn id="13" name="Tổng tiền trả (VND)"/>
-    <x:tableColumn id="14" name="Khách hàng"/>
-    <x:tableColumn id="15" name="Tình trạng"/>
-    <x:tableColumn id="16" name="Đối chiếu sổ AMIS 2024"/>
-    <x:tableColumn id="17" name="Dòng sổ AMIS"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -10972,7 +10933,9 @@
       <x:c r="B196" s="6" t="d">
         <x:v>2024-12-03T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C196" s="7" t="str"/>
+      <x:c r="C196" s="7" t="str">
+        <x:v>BHHT2024024972</x:v>
+      </x:c>
       <x:c r="D196" s="2" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -11008,7 +10971,7 @@
         <x:v>Khách hàng Tiktok</x:v>
       </x:c>
       <x:c r="O196" s="2" t="str">
-        <x:v>Trống BHH trên AMIS</x:v>
+        <x:v>BHH do người dùng xác nhận 2026-10-27; AMIS lúc trích đang trống</x:v>
       </x:c>
       <x:c r="P196" s="2" t="str">
         <x:v>Khớp sổ AMIS 2024</x:v>
@@ -12319,7 +12282,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87684e12202a4454"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9341ab71559d4682"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12356,7 +12319,7 @@
         <x:v>Số dòng hàng</x:v>
       </x:c>
       <x:c r="E1" s="5" t="str">
-        <x:v>BHH gốc trên AMIS</x:v>
+        <x:v>BHH gốc đã xác định</x:v>
       </x:c>
       <x:c r="F1" s="5" t="str">
         <x:v>Số lượng trả</x:v>
@@ -18628,7 +18591,9 @@
       <x:c r="D147" s="2" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E147" s="10" t="str"/>
+      <x:c r="E147" s="10" t="str">
+        <x:v>BHHT2024024972</x:v>
+      </x:c>
       <x:c r="F147" s="11" t="n">
         <x:f>SUM('Chi tiet BTL-BHH'!H196:H196)</x:f>
         <x:v>1</x:v>
@@ -19395,7 +19360,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe93eb31c5624901"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7e561244bf94786"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19463,7 +19428,7 @@
         <x:v>Số BHH gốc khác nhau</x:v>
       </x:c>
       <x:c r="B7" s="10" t="n">
-        <x:v>162</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
@@ -19471,7 +19436,7 @@
         <x:v>Số dòng trống BHH</x:v>
       </x:c>
       <x:c r="B8" s="10" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
@@ -19522,7 +19487,7 @@
         <x:v>Phương pháp</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>Đọc trực tiếp từng phiếu và từng dòng hàng trên AMIS. Kiểm đủ dòng và tổng tiền, đối chiếu từng dòng với sổ AMIS 2024.</x:v>
+        <x:v>Đọc trực tiếp AMIS, kiểm đủ dòng/tổng tiền và đối chiếu sổ AMIS 2024. Bổ sung riêng BTL00145 → BHHT2024024972 theo xác nhận người dùng 27/10/2026; giữ nguyên snapshot đọc AMIS ban đầu.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
@@ -19530,7 +19495,7 @@
         <x:v>Ý nghĩa BHH</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>Giữ nguyên BHH do AMIS hiển thị, không suy đoán theo tên, số tiền hay đơn giá.</x:v>
+        <x:v>BHH lấy từ AMIS; riêng BTL00145 do người dùng xác nhận. Nguồn liên kết ghi rõ ở cột Liên kết trên AMIS. Không suy đoán theo tên/giá.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
@@ -19559,152 +19524,16 @@
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="2" t="str">
-        <x:v>Phiếu cần kiểm tra</x:v>
+        <x:v>Liên kết bổ sung</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>BTL00145 / SP000042 đang trống Số CT bán hàng trên AMIS; giữ nguyên trống, xem Chua co BHH.</x:v>
+        <x:v>BTL00145 / SP000042 → BHHT2024024972 do người dùng xác nhận 27/10/2026. Snapshot AMIS lúc trích vẫn trống. SL, đơn giá, tiền hàng/VAT/thanh toán khớp hoàn toàn, trả hết.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d3e717c6e3a46ee"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="85" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="25" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="21" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="25" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="27" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="34" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="27" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="32" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="44" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Số phiếu BTL</x:v>
-      </x:c>
-      <x:c r="B1" s="5" t="str">
-        <x:v>Ngày hạch toán</x:v>
-      </x:c>
-      <x:c r="C1" s="5" t="str">
-        <x:v>BHH gốc đang trống</x:v>
-      </x:c>
-      <x:c r="D1" s="5" t="str">
-        <x:v>Dòng BTL</x:v>
-      </x:c>
-      <x:c r="E1" s="5" t="str">
-        <x:v>Mã hàng</x:v>
-      </x:c>
-      <x:c r="F1" s="5" t="str">
-        <x:v>Tên hàng</x:v>
-      </x:c>
-      <x:c r="G1" s="5" t="str">
-        <x:v>ĐVT</x:v>
-      </x:c>
-      <x:c r="H1" s="5" t="str">
-        <x:v>Số lượng trả</x:v>
-      </x:c>
-      <x:c r="I1" s="5" t="str">
-        <x:v>Đơn giá (VND)</x:v>
-      </x:c>
-      <x:c r="J1" s="5" t="str">
-        <x:v>Tiền hàng trả (VND)</x:v>
-      </x:c>
-      <x:c r="K1" s="5" t="str">
-        <x:v>Thuế suất GTGT (%)</x:v>
-      </x:c>
-      <x:c r="L1" s="5" t="str">
-        <x:v>Tiền thuế GTGT (VND)</x:v>
-      </x:c>
-      <x:c r="M1" s="5" t="str">
-        <x:v>Tổng tiền trả (VND)</x:v>
-      </x:c>
-      <x:c r="N1" s="5" t="str">
-        <x:v>Khách hàng</x:v>
-      </x:c>
-      <x:c r="O1" s="5" t="str">
-        <x:v>Tình trạng</x:v>
-      </x:c>
-      <x:c r="P1" s="5" t="str">
-        <x:v>Đối chiếu sổ AMIS 2024</x:v>
-      </x:c>
-      <x:c r="Q1" s="5" t="str">
-        <x:v>Dòng sổ AMIS</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="42" customHeight="1">
-      <x:c r="A2" s="2" t="str">
-        <x:v>BTL00145</x:v>
-      </x:c>
-      <x:c r="B2" s="6" t="d">
-        <x:v>2024-12-03T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C2" s="13" t="str"/>
-      <x:c r="D2" s="2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" s="2" t="str">
-        <x:v>SP000042</x:v>
-      </x:c>
-      <x:c r="F2" s="10" t="str">
-        <x:v>Bình nước giữ nhiệt thông minh UVGREEN UK100 Màu trắng</x:v>
-      </x:c>
-      <x:c r="G2" s="2" t="str">
-        <x:v>Cái</x:v>
-      </x:c>
-      <x:c r="H2" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I2" s="8" t="n">
-        <x:v>972222</x:v>
-      </x:c>
-      <x:c r="J2" s="14" t="n">
-        <x:v>972222</x:v>
-      </x:c>
-      <x:c r="K2" s="14" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="L2" s="14" t="n">
-        <x:v>77778</x:v>
-      </x:c>
-      <x:c r="M2" s="14" t="n">
-        <x:f>J2+L2</x:f>
-        <x:v>1050000</x:v>
-      </x:c>
-      <x:c r="N2" s="2" t="str">
-        <x:v>Khách hàng Tiktok</x:v>
-      </x:c>
-      <x:c r="O2" s="2" t="str">
-        <x:v>Trống BHH trên AMIS</x:v>
-      </x:c>
-      <x:c r="P2" s="2" t="str">
-        <x:v>Khớp sổ AMIS 2024</x:v>
-      </x:c>
-      <x:c r="Q2" s="2" t="str">
-        <x:v>40633</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fce768deab74237"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6bdfbdd082d4e8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>